<commit_message>
Fill in start prices, deposits and auction steps in tender registry
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZUCsNNmeJ2qjAHjE6D5fq
</commit_message>
<xml_diff>
--- a/reestr_torgi.xlsx
+++ b/reestr_torgi.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Реестр" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Реестр!$A$4:$AG$13</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Реестр!$A$4:$AJ$13</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,59 +22,13 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <authors>
-    <author>Unknown Author</author>
-  </authors>
-  <commentList>
-    <comment ref="Q9" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Цена, задаток и шаг из публикации РБК Недвижимости (finance.mail.ru, 18.09.2026) со ссылкой на инвестпортал Москвы. В карточке цена не отображается.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q12" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Каталог investmoscow.ru, раздел «Купить здание», 20.10.2026: 195 014 000 ₽ (307 399,12 ₽ за м²).</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q13" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Каталог investmoscow.ru, раздел «Купить здание», 20.10.2026: 158 898 000 ₽ (176 887,45 ₽ за м²).</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="134">
   <si>
     <t xml:space="preserve">Реестр объектов торгов (investmoscow.ru / roseltorg.ru)</t>
   </si>
   <si>
-    <t xml:space="preserve">Данные собраны 20.10.2026 с карточек investmoscow.ru. Розовая ячейка «н/д» — цена на странице не опубликована в доступном виде или площадка недоступна (см. примечания).</t>
+    <t xml:space="preserve">Собрано 20.10.2026 из карточек investmoscow.ru (блок «О процедуре»). Время московское. «н/д» — данные недоступны (см. примечание).</t>
   </si>
   <si>
     <t xml:space="preserve">№</t>
@@ -137,6 +91,15 @@
     <t xml:space="preserve">Шаг аукциона, ₽</t>
   </si>
   <si>
+    <t xml:space="preserve">Форма торгов</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Процедура на ЭТП</t>
+  </si>
+  <si>
+    <t xml:space="preserve">torgi.gov.ru</t>
+  </si>
+  <si>
     <t xml:space="preserve">Кадастровый № объекта</t>
   </si>
   <si>
@@ -158,19 +121,19 @@
     <t xml:space="preserve">ОКН</t>
   </si>
   <si>
-    <t xml:space="preserve">Приём заявок с</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Приём заявок до</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Отбор участников</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Проведение торгов</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Подведение итогов</t>
+    <t xml:space="preserve">Приём заявок с (МСК)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Приём заявок до (МСК)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отбор участников (МСК)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Проведение торгов (МСК)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Подведение итогов (МСК)</t>
   </si>
   <si>
     <t xml:space="preserve">Примечание</t>
@@ -188,15 +151,12 @@
     <t xml:space="preserve">н/д</t>
   </si>
   <si>
-    <t xml:space="preserve">Roseltorg недоступен из среды сбора (соединение сбрасывается, 503). Номер похож на извещение torgi.gov.ru, но он тоже недоступен. Данные нужно внести вручную.</t>
+    <t xml:space="preserve">Roseltorg и torgi.gov.ru блокируют запросы не из РФ — страница недоступна ни напрямую, ни через сервисы-посредники. Данные нужно внести вручную.</t>
   </si>
   <si>
     <t xml:space="preserve">COM13102600087</t>
   </si>
   <si>
-    <t xml:space="preserve">Roseltorg недоступен из среды сбора (соединение сбрасывается, 503). Данные нужно внести вручную.</t>
-  </si>
-  <si>
     <t xml:space="preserve">investmoscow.ru</t>
   </si>
   <si>
@@ -227,6 +187,15 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
+    <t xml:space="preserve">Открытый аукцион в электронной форме</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roseltorg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">извещение</t>
+  </si>
+  <si>
     <t xml:space="preserve">77:01:0001033:2521</t>
   </si>
   <si>
@@ -239,22 +208,22 @@
     <t xml:space="preserve">Нет</t>
   </si>
   <si>
-    <t xml:space="preserve">14.09.2026 17:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09.11.2026 12:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16.11.2026 07:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.11.2026 07:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.11.2026 14:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Цена подгружается на сайте скриптом и в доступной версии страницы отсутствует. Район указан по адресному справочнику, а не по карточке.</t>
+    <t xml:space="preserve">14.09.2026 20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09.11.2026 15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.11.2026 10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.11.2026 10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.11.2026 17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Район указан по адресному справочнику (в карточке не указан).</t>
   </si>
   <si>
     <t xml:space="preserve">20212872</t>
@@ -278,22 +247,22 @@
     <t xml:space="preserve">Да</t>
   </si>
   <si>
-    <t xml:space="preserve">13.10.2026 17:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16.11.2026 12:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19.11.2026 07:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.11.2026 07:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24.11.2026 14:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Цена подгружается на сайте скриптом и в доступной версии страницы отсутствует. Объект культурного наследия.</t>
+    <t xml:space="preserve">13.10.2026 20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.11.2026 15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19.11.2026 10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.11.2026 10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24.11.2026 17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Объект культурного наследия.</t>
   </si>
   <si>
     <t xml:space="preserve">20182722</t>
@@ -317,19 +286,19 @@
     <t xml:space="preserve">77:01:0002018:1071</t>
   </si>
   <si>
-    <t xml:space="preserve">17.09.2026 17:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13.11.2026 12:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20.11.2026 07:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20.11.2026 14:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">В списке ссылок указан дважды. Цена, задаток и шаг взяты из СМИ, где были другие даты (заявки до 26.10, торги 06.11). Сроки, видимо, продлили; цену стоит сверить с извещением. Объект культурного наследия.</t>
+    <t xml:space="preserve">17.09.2026 20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.11.2026 15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.11.2026 10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.11.2026 17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В вашем списке ссылка была дважды. Вид цены — «плата за право заключения договора купли-продажи». Процедура по 178-ФЗ, ссылки на torgi.gov.ru в карточке нет. Объект культурного наследия.</t>
   </si>
   <si>
     <t xml:space="preserve">20202772</t>
@@ -353,10 +322,10 @@
     <t xml:space="preserve">Через иную собственность</t>
   </si>
   <si>
-    <t xml:space="preserve">24.09.2026 17:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11.11.2026 12:00</t>
+    <t xml:space="preserve">24.09.2026 20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.11.2026 15:00</t>
   </si>
   <si>
     <t xml:space="preserve">20208821</t>
@@ -377,19 +346,16 @@
     <t xml:space="preserve">Через подъезд</t>
   </si>
   <si>
-    <t xml:space="preserve">06.10.2026 17:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.11.2026 07:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.11.2026 07:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.11.2026 14:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Цена подгружается на сайте скриптом и в доступной версии страницы отсутствует.</t>
+    <t xml:space="preserve">06.10.2026 20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.11.2026 10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.11.2026 10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.11.2026 17:00</t>
   </si>
   <si>
     <t xml:space="preserve">20209390</t>
@@ -416,7 +382,7 @@
     <t xml:space="preserve">77:01:0001080:2978</t>
   </si>
   <si>
-    <t xml:space="preserve">07.10.2026 17:00</t>
+    <t xml:space="preserve">07.10.2026 20:00</t>
   </si>
   <si>
     <t xml:space="preserve">Цена за м² считается по площади здания.</t>
@@ -449,16 +415,16 @@
     <t xml:space="preserve">Итого (средняя цена за м² — по объектам с известной ценой)</t>
   </si>
   <si>
-    <t xml:space="preserve">Источник: карточки investmoscow.ru (собраны 20.10.2026). Цены зданий на Неглинной и Каширском шоссе взяты из каталога investmoscow.ru; цена на Пятницкой взята из СМИ (подробнее в комментарии к ячейке).</t>
+    <t xml:space="preserve">Источник: карточки investmoscow.ru, блок «О процедуре» (начальная цена, задаток, шаг, сроки, ссылки на ЭТП и torgi.gov.ru), по состоянию на 20.10.2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Ссылка investmoscow.ru/tenders/tender/20182722 повторялась в списке дважды, в реестре она одна строка.</t>
   </si>
   <si>
-    <t xml:space="preserve">«Цена за м²» и строка «Итого» считаются формулами: после ввода недостающих цен они пересчитаются сами.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Площадь ЗУ для зданий указана по заголовку карточки (в поле «Площадь земельного участка» стоит «Не указано»).</t>
+    <t xml:space="preserve">«Цена за м²» и строка «Итого» считаются формулами: после ввода цен по лотам roseltorg они пересчитаются сами.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Площадь ЗУ для зданий взята из заголовка карточки (в поле «Площадь земельного участка» стоит «Не указано»).</t>
   </si>
 </sst>
 </file>
@@ -471,7 +437,7 @@
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="#,##0&quot; ₽&quot;"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -551,11 +517,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -981,7 +942,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AG19"/>
+  <dimension ref="A1:AJ19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1003,13 +964,15 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="21" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="25" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="28" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="22" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="24" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="28" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="31" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1122,19 +1085,28 @@
       <c r="AG4" s="3" t="s">
         <v>34</v>
       </c>
+      <c r="AH4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AI4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="AJ4" s="3" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
@@ -1149,7 +1121,7 @@
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="R5" s="9" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q5),ISNUMBER(M5),M5&gt;0),Q5/M5,"")</f>
@@ -1169,22 +1141,25 @@
       <c r="AD5" s="4"/>
       <c r="AE5" s="4"/>
       <c r="AF5" s="4"/>
-      <c r="AG5" s="4" t="s">
-        <v>39</v>
+      <c r="AG5" s="4"/>
+      <c r="AH5" s="4"/>
+      <c r="AI5" s="4"/>
+      <c r="AJ5" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
@@ -1199,7 +1174,7 @@
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="R6" s="9" t="str">
         <f aca="false">IF(AND(ISNUMBER(Q6),ISNUMBER(M6),M6&gt;0),Q6/M6,"")</f>
@@ -1219,43 +1194,46 @@
       <c r="AD6" s="4"/>
       <c r="AE6" s="4"/>
       <c r="AF6" s="4"/>
-      <c r="AG6" s="4" t="s">
-        <v>41</v>
+      <c r="AG6" s="4"/>
+      <c r="AH6" s="4"/>
+      <c r="AI6" s="4"/>
+      <c r="AJ6" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="L7" s="4" t="n">
         <v>5</v>
@@ -1265,91 +1243,104 @@
       </c>
       <c r="N7" s="7"/>
       <c r="O7" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="P7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="Q7" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="R7" s="9" t="str">
+      <c r="Q7" s="9" t="n">
+        <v>15384000</v>
+      </c>
+      <c r="R7" s="9" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q7),ISNUMBER(M7),M7&gt;0),Q7/M7,"")</f>
-        <v/>
-      </c>
-      <c r="S7" s="9"/>
-      <c r="T7" s="9"/>
+        <v>363687.943262411</v>
+      </c>
+      <c r="S7" s="9" t="n">
+        <v>1538400</v>
+      </c>
+      <c r="T7" s="9" t="n">
+        <v>769200</v>
+      </c>
       <c r="U7" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="V7" s="4"/>
-      <c r="W7" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="X7" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="Y7" s="4" t="s">
-        <v>55</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="Y7" s="4"/>
       <c r="Z7" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="AA7" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="AB7" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="AC7" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD7" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="AE7" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AF7" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="AG7" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
+      </c>
+      <c r="AH7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="AI7" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ7" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>9</v>
@@ -1359,54 +1350,67 @@
       </c>
       <c r="N8" s="7"/>
       <c r="O8" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="P8" s="4"/>
-      <c r="Q8" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="R8" s="9" t="str">
+      <c r="Q8" s="9" t="n">
+        <v>239527000</v>
+      </c>
+      <c r="R8" s="9" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q8),ISNUMBER(M8),M8&gt;0),Q8/M8,"")</f>
-        <v/>
-      </c>
-      <c r="S8" s="9"/>
-      <c r="T8" s="9"/>
+        <v>555489.332096475</v>
+      </c>
+      <c r="S8" s="9" t="n">
+        <v>47905400</v>
+      </c>
+      <c r="T8" s="9" t="n">
+        <v>2395270</v>
+      </c>
       <c r="U8" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="V8" s="4"/>
-      <c r="W8" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="X8" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y8" s="4" t="s">
-        <v>55</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="Y8" s="4"/>
       <c r="Z8" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="AA8" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="AB8" s="4" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="AC8" s="4" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="AD8" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="AE8" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="AF8" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="AG8" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
+      </c>
+      <c r="AH8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="AI8" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="AJ8" s="4" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1414,34 +1418,34 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="L9" s="4" t="n">
         <v>2</v>
@@ -1465,77 +1469,84 @@
         <v>131500000</v>
       </c>
       <c r="T9" s="9" t="n">
-        <v>2600000</v>
+        <v>2630000</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="V9" s="4"/>
-      <c r="W9" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="X9" s="4"/>
-      <c r="Y9" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="V9" s="5" t="s">
         <v>55</v>
       </c>
+      <c r="W9" s="4"/>
+      <c r="X9" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y9" s="4"/>
       <c r="Z9" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="AA9" s="4" t="s">
-        <v>68</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="AA9" s="4"/>
       <c r="AB9" s="4" t="s">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="AC9" s="4" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="AD9" s="4" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="AE9" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="AF9" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="AG9" s="4" t="s">
-        <v>86</v>
+        <v>64</v>
+      </c>
+      <c r="AH9" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="AI9" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="AJ9" s="4" t="s">
+        <v>91</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>9</v>
@@ -1545,56 +1556,69 @@
       </c>
       <c r="N10" s="7"/>
       <c r="O10" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="Q10" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="R10" s="9" t="str">
+      <c r="Q10" s="9" t="n">
+        <v>17225000</v>
+      </c>
+      <c r="R10" s="9" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q10),ISNUMBER(M10),M10&gt;0),Q10/M10,"")</f>
-        <v/>
-      </c>
-      <c r="S10" s="9"/>
-      <c r="T10" s="9"/>
+        <v>1314885.49618321</v>
+      </c>
+      <c r="S10" s="9" t="n">
+        <v>1722500</v>
+      </c>
+      <c r="T10" s="9" t="n">
+        <v>861250</v>
+      </c>
       <c r="U10" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="V10" s="4"/>
-      <c r="W10" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="V10" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="W10" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="X10" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="Y10" s="4" t="s">
-        <v>55</v>
-      </c>
+        <v>97</v>
+      </c>
+      <c r="Y10" s="4"/>
       <c r="Z10" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="AA10" s="4" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="AB10" s="4" t="s">
-        <v>94</v>
+        <v>60</v>
       </c>
       <c r="AC10" s="4" t="s">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="AD10" s="4" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="AE10" s="4" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="AF10" s="4" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="AG10" s="4" t="s">
-        <v>74</v>
+        <v>64</v>
+      </c>
+      <c r="AH10" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="AI10" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="AJ10" s="4" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1602,34 +1626,34 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L11" s="4" t="n">
         <v>9</v>
@@ -1639,91 +1663,102 @@
       </c>
       <c r="N11" s="7"/>
       <c r="O11" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="P11" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q11" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="R11" s="9" t="str">
+      <c r="Q11" s="9" t="n">
+        <v>50797000</v>
+      </c>
+      <c r="R11" s="9" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q11),ISNUMBER(M11),M11&gt;0),Q11/M11,"")</f>
-        <v/>
-      </c>
-      <c r="S11" s="9"/>
-      <c r="T11" s="9"/>
+        <v>303991.621783363</v>
+      </c>
+      <c r="S11" s="9" t="n">
+        <v>5079700</v>
+      </c>
+      <c r="T11" s="9" t="n">
+        <v>2539850</v>
+      </c>
       <c r="U11" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="V11" s="4"/>
-      <c r="W11" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="V11" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="W11" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="X11" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="Y11" s="4" t="s">
-        <v>55</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="Y11" s="4"/>
       <c r="Z11" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="AA11" s="4" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
       <c r="AB11" s="4" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="AC11" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD11" s="4" t="s">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="AE11" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="AF11" s="4" t="s">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="AG11" s="4" t="s">
-        <v>106</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="AH11" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="AI11" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="AJ11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>4</v>
@@ -1745,44 +1780,57 @@
         <f aca="false">IF(AND(ISNUMBER(Q12),ISNUMBER(M12),M12&gt;0),Q12/M12,"")</f>
         <v>307399.117276166</v>
       </c>
-      <c r="S12" s="9"/>
-      <c r="T12" s="9"/>
+      <c r="S12" s="9" t="n">
+        <v>39002800</v>
+      </c>
+      <c r="T12" s="9" t="n">
+        <v>1950140</v>
+      </c>
       <c r="U12" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="V12" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="W12" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="X12" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="V12" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="W12" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="X12" s="4" t="s">
+        <v>117</v>
+      </c>
       <c r="Y12" s="4" t="s">
-        <v>55</v>
+        <v>118</v>
       </c>
       <c r="Z12" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="AA12" s="4" t="s">
-        <v>55</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="AA12" s="4"/>
       <c r="AB12" s="4" t="s">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="AC12" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD12" s="4" t="s">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="AE12" s="4" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="AF12" s="4" t="s">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="AG12" s="4" t="s">
-        <v>116</v>
+        <v>108</v>
+      </c>
+      <c r="AH12" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="AI12" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="AJ12" s="4" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1790,34 +1838,34 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="L13" s="4" t="n">
         <v>12</v>
@@ -1839,49 +1887,62 @@
         <f aca="false">IF(AND(ISNUMBER(Q13),ISNUMBER(M13),M13&gt;0),Q13/M13,"")</f>
         <v>176887.454079929</v>
       </c>
-      <c r="S13" s="9"/>
-      <c r="T13" s="9"/>
+      <c r="S13" s="9" t="n">
+        <v>31779600</v>
+      </c>
+      <c r="T13" s="9" t="n">
+        <v>1588980</v>
+      </c>
       <c r="U13" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="V13" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="W13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="X13" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="V13" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="W13" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="X13" s="4" t="s">
+        <v>127</v>
+      </c>
       <c r="Y13" s="4" t="s">
-        <v>55</v>
+        <v>128</v>
       </c>
       <c r="Z13" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="AA13" s="4" t="s">
-        <v>55</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="AA13" s="4"/>
       <c r="AB13" s="4" t="s">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="AC13" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD13" s="4" t="s">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="AE13" s="4" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="AF13" s="4" t="s">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="AG13" s="4" t="s">
-        <v>116</v>
+        <v>108</v>
+      </c>
+      <c r="AH13" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="AI13" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="AJ13" s="4" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J14" s="10" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="M14" s="11" t="n">
         <f aca="false">SUM(M5:M13)</f>
@@ -1889,45 +1950,58 @@
       </c>
       <c r="Q14" s="12" t="n">
         <f aca="false">SUM(Q5:Q13)</f>
-        <v>616912000</v>
+        <v>939845000</v>
       </c>
       <c r="R14" s="12" t="n">
         <f aca="false">IFERROR(SUM(Q5:Q13)/SUMIF(Q5:Q13,"&gt;0",M5:M13),"")</f>
-        <v>240717.964726081</v>
+        <v>292194.932379916</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AG13"/>
+  <autoFilter ref="A4:AJ13"/>
   <hyperlinks>
-    <hyperlink ref="C5" r:id="rId2" display="открыть"/>
-    <hyperlink ref="C6" r:id="rId3" display="открыть"/>
-    <hyperlink ref="C7" r:id="rId4" display="открыть"/>
-    <hyperlink ref="C8" r:id="rId5" display="открыть"/>
-    <hyperlink ref="C9" r:id="rId6" display="открыть"/>
-    <hyperlink ref="C10" r:id="rId7" display="открыть"/>
-    <hyperlink ref="C11" r:id="rId8" display="открыть"/>
-    <hyperlink ref="C12" r:id="rId9" display="открыть"/>
-    <hyperlink ref="C13" r:id="rId10" display="открыть"/>
+    <hyperlink ref="C5" r:id="rId1" display="открыть"/>
+    <hyperlink ref="C6" r:id="rId2" display="открыть"/>
+    <hyperlink ref="C7" r:id="rId3" display="открыть"/>
+    <hyperlink ref="V7" r:id="rId4" display="roseltorg"/>
+    <hyperlink ref="W7" r:id="rId5" display="извещение"/>
+    <hyperlink ref="C8" r:id="rId6" display="открыть"/>
+    <hyperlink ref="V8" r:id="rId7" display="roseltorg"/>
+    <hyperlink ref="W8" r:id="rId8" display="извещение"/>
+    <hyperlink ref="C9" r:id="rId9" display="открыть"/>
+    <hyperlink ref="V9" r:id="rId10" display="roseltorg"/>
+    <hyperlink ref="C10" r:id="rId11" display="открыть"/>
+    <hyperlink ref="V10" r:id="rId12" display="roseltorg"/>
+    <hyperlink ref="W10" r:id="rId13" display="извещение"/>
+    <hyperlink ref="C11" r:id="rId14" display="открыть"/>
+    <hyperlink ref="V11" r:id="rId15" display="roseltorg"/>
+    <hyperlink ref="W11" r:id="rId16" display="извещение"/>
+    <hyperlink ref="C12" r:id="rId17" display="открыть"/>
+    <hyperlink ref="V12" r:id="rId18" display="roseltorg"/>
+    <hyperlink ref="W12" r:id="rId19" display="извещение"/>
+    <hyperlink ref="C13" r:id="rId20" display="открыть"/>
+    <hyperlink ref="V13" r:id="rId21" display="roseltorg"/>
+    <hyperlink ref="W13" r:id="rId22" display="извещение"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1936,7 +2010,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId11"/>
-  <legacyDrawing r:id="rId12"/>
+  <drawing r:id="rId23"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add roseltorg lots (Krasnoprudnaya 3B, Bolshaya Sukharevskaya 1/2) to tender registry
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZUCsNNmeJ2qjAHjE6D5fq
</commit_message>
<xml_diff>
--- a/reestr_torgi.xlsx
+++ b/reestr_torgi.xlsx
@@ -22,13 +22,35 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="Q6" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Площадь 315,5 м² взята из объявления Абсолют Банка на ЦИАН (та же цена — 112,95 млн ₽, с НДС 22%). На странице roseltorg площадь не указана — она есть только в аукционной документации (.doc).</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="134">
-  <si>
-    <t xml:space="preserve">Реестр объектов торгов (investmoscow.ru / roseltorg.ru)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Собрано 20.10.2026 из карточек investmoscow.ru (блок «О процедуре»). Время московское. «н/д» — данные недоступны (см. примечание).</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="155">
+  <si>
+    <t xml:space="preserve">Реестр объектов торгов, Москва (investmoscow.ru / roseltorg.ru)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Собрано 20.10.2026: карточки investmoscow.ru (блок «О процедуре»), процедуры roseltorg.ru, извещение torgi.gov.ru. Время московское.</t>
   </si>
   <si>
     <t xml:space="preserve">№</t>
@@ -148,15 +170,99 @@
     <t xml:space="preserve">21000003370000000430</t>
   </si>
   <si>
-    <t xml:space="preserve">н/д</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roseltorg и torgi.gov.ru блокируют запросы не из РФ — страница недоступна ни напрямую, ни через сервисы-посредники. Данные нужно внести вручную.</t>
+    <t xml:space="preserve">Здание + земельный участок</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Продажа</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ЦАО</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Красносельский</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Краснопрудная ул., д. 3Б (земельный участок 3/5/1), здание Ярославского ПЖДП</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Красносельская</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Электронный аукцион на повышение (178-ФЗ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roseltorg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">извещение</t>
+  </si>
+  <si>
+    <t xml:space="preserve">77:01:0003036:1085</t>
+  </si>
+  <si>
+    <t xml:space="preserve">77:01:0003036:4449</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Услуги связи (ВРИ участка 3.2.3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">По выписке ЕГРН</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.10.2026 20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25.11.2026 23:59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">до 27.11.2026 23:59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30.11.2026 11:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Продавец — АО «Почта России», организатор — АО ИФК «Солид». Продаётся единым лотом: здание 1 259,3 м² и участок 621 ± 9 м² (общая площадь 1 880,3 м²). Задаток 20%. Цена, задаток и шаг указаны в извещении torgi.gov.ru (данные взяты с зеркала torgi-ru.com, лот 8152317).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roseltorg.ru (com)</t>
   </si>
   <si>
     <t xml:space="preserve">COM13102600087</t>
   </si>
   <si>
+    <t xml:space="preserve">Нежилое помещение</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Мещанский</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Большая Сухаревская пл., д. 1/2, стр. 1, помещ. 3/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сухаревская</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Подвал, 1 этаж, антресоль</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Аукцион на повышение (коммерческая процедура)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.10.2026 14:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.12.2026 14:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.12.2026 15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.12.2026 11:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Продавец и организатор — АКБ «Абсолют Банк» (ПАО). Задаток — обеспечение заявки 10%. Шаг аукциона на странице не указан (он в аукционной документации). Цена с НДС 22%. Первая линия Садового кольца, 20 м от выхода метро.</t>
+  </si>
+  <si>
     <t xml:space="preserve">investmoscow.ru</t>
   </si>
   <si>
@@ -166,15 +272,6 @@
     <t xml:space="preserve">17003139</t>
   </si>
   <si>
-    <t xml:space="preserve">Нежилое помещение</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Продажа</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ЦАО</t>
-  </si>
-  <si>
     <t xml:space="preserve">Басманный</t>
   </si>
   <si>
@@ -190,12 +287,6 @@
     <t xml:space="preserve">Открытый аукцион в электронной форме</t>
   </si>
   <si>
-    <t xml:space="preserve">roseltorg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">извещение</t>
-  </si>
-  <si>
     <t xml:space="preserve">77:01:0001033:2521</t>
   </si>
   <si>
@@ -364,12 +455,6 @@
     <t xml:space="preserve">17007468</t>
   </si>
   <si>
-    <t xml:space="preserve">Здание + земельный участок</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Мещанский</t>
-  </si>
-  <si>
     <t xml:space="preserve">Неглинная ул., д. 18/1, стр. 2</t>
   </si>
   <si>
@@ -415,13 +500,13 @@
     <t xml:space="preserve">Итого (средняя цена за м² — по объектам с известной ценой)</t>
   </si>
   <si>
-    <t xml:space="preserve">Источник: карточки investmoscow.ru, блок «О процедуре» (начальная цена, задаток, шаг, сроки, ссылки на ЭТП и torgi.gov.ru), по состоянию на 20.10.2026.</t>
+    <t xml:space="preserve">Источники: карточки investmoscow.ru (блок «О процедуре»), страницы процедур roseltorg.ru, извещение torgi.gov.ru 21000003370000000430 (через зеркало torgi-ru.com) и объявление Абсолют Банка на ЦИАН (площадь лота COM13102600087). Состояние на 20.10.2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Ссылка investmoscow.ru/tenders/tender/20182722 повторялась в списке дважды, в реестре она одна строка.</t>
   </si>
   <si>
-    <t xml:space="preserve">«Цена за м²» и строка «Итого» считаются формулами: после ввода цен по лотам roseltorg они пересчитаются сами.</t>
+    <t xml:space="preserve">«Цена за м²» и строка «Итого» считаются формулами.</t>
   </si>
   <si>
     <t xml:space="preserve">Площадь ЗУ для зданий взята из заголовка карточки (в поле «Площадь земельного участка» стоит «Не указано»).</t>
@@ -431,13 +516,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="#,##0&quot; ₽&quot;"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00&quot; ₽&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -518,8 +604,13 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -530,12 +621,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
         <bgColor rgb="FF333333"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4D6"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -621,11 +706,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -654,7 +739,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -686,14 +771,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE4D6"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <colors>
     <indexedColors>
@@ -715,7 +792,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFCE4D6"/>
+      <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -1095,7 +1172,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -1109,81 +1186,153 @@
         <v>40</v>
       </c>
       <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="7"/>
+      <c r="F5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>1259.3</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>621</v>
+      </c>
       <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="R5" s="9" t="str">
+      <c r="P5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="8" t="n">
+        <v>289558721</v>
+      </c>
+      <c r="R5" s="8" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q5),ISNUMBER(M5),M5&gt;0),Q5/M5,"")</f>
-        <v/>
-      </c>
-      <c r="S5" s="9"/>
-      <c r="T5" s="9"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="4"/>
-      <c r="Y5" s="4"/>
-      <c r="Z5" s="4"/>
+        <v>229936.251091876</v>
+      </c>
+      <c r="S5" s="9" t="n">
+        <v>57911744.2</v>
+      </c>
+      <c r="T5" s="9" t="n">
+        <v>5791174.42</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="X5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z5" s="4" t="s">
+        <v>52</v>
+      </c>
       <c r="AA5" s="4"/>
       <c r="AB5" s="4"/>
-      <c r="AC5" s="4"/>
+      <c r="AC5" s="4" t="s">
+        <v>53</v>
+      </c>
       <c r="AD5" s="4"/>
-      <c r="AE5" s="4"/>
-      <c r="AF5" s="4"/>
-      <c r="AG5" s="4"/>
-      <c r="AH5" s="4"/>
+      <c r="AE5" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AG5" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH5" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="AI5" s="4"/>
       <c r="AJ5" s="4" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="6"/>
+      <c r="I6" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>315.5</v>
+      </c>
       <c r="N6" s="7"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="R6" s="9" t="str">
+      <c r="O6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="8" t="n">
+        <v>112951260</v>
+      </c>
+      <c r="R6" s="8" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q6),ISNUMBER(M6),M6&gt;0),Q6/M6,"")</f>
-        <v/>
-      </c>
-      <c r="S6" s="9"/>
+        <v>358007.163232964</v>
+      </c>
+      <c r="S6" s="9" t="n">
+        <v>11295126</v>
+      </c>
       <c r="T6" s="9"/>
-      <c r="U6" s="4"/>
-      <c r="V6" s="4"/>
+      <c r="U6" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="W6" s="4"/>
       <c r="X6" s="4"/>
       <c r="Y6" s="4"/>
@@ -1192,13 +1341,21 @@
       <c r="AB6" s="4"/>
       <c r="AC6" s="4"/>
       <c r="AD6" s="4"/>
-      <c r="AE6" s="4"/>
-      <c r="AF6" s="4"/>
-      <c r="AG6" s="4"/>
-      <c r="AH6" s="4"/>
+      <c r="AE6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AG6" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AH6" s="4" t="s">
+        <v>70</v>
+      </c>
       <c r="AI6" s="4"/>
       <c r="AJ6" s="4" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1206,34 +1363,34 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>52</v>
+        <v>77</v>
       </c>
       <c r="L7" s="4" t="n">
         <v>5</v>
@@ -1243,15 +1400,15 @@
       </c>
       <c r="N7" s="7"/>
       <c r="O7" s="4" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="P7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="Q7" s="9" t="n">
+      <c r="Q7" s="8" t="n">
         <v>15384000</v>
       </c>
-      <c r="R7" s="9" t="n">
+      <c r="R7" s="8" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q7),ISNUMBER(M7),M7&gt;0),Q7/M7,"")</f>
         <v>363687.943262411</v>
       </c>
@@ -1262,50 +1419,50 @@
         <v>769200</v>
       </c>
       <c r="U7" s="4" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="V7" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="X7" s="4" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="Y7" s="4"/>
       <c r="Z7" s="4" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="AA7" s="4" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="AB7" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AC7" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AD7" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AE7" s="4" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="AF7" s="4" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="AG7" s="4" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="AH7" s="4" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="AI7" s="4" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="AJ7" s="4" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1313,34 +1470,34 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>9</v>
@@ -1350,13 +1507,13 @@
       </c>
       <c r="N8" s="7"/>
       <c r="O8" s="4" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="P8" s="4"/>
-      <c r="Q8" s="9" t="n">
+      <c r="Q8" s="8" t="n">
         <v>239527000</v>
       </c>
-      <c r="R8" s="9" t="n">
+      <c r="R8" s="8" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q8),ISNUMBER(M8),M8&gt;0),Q8/M8,"")</f>
         <v>555489.332096475</v>
       </c>
@@ -1367,50 +1524,50 @@
         <v>2395270</v>
       </c>
       <c r="U8" s="4" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="V8" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="X8" s="4" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="Y8" s="4"/>
       <c r="Z8" s="4" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="AA8" s="4" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="AB8" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AC8" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AD8" s="4" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="AE8" s="4" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="AF8" s="4" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="AG8" s="4" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="AH8" s="4" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="AI8" s="4" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="AJ8" s="4" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1418,34 +1575,34 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="L9" s="4" t="n">
         <v>2</v>
@@ -1458,10 +1615,10 @@
       <c r="P9" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="Q9" s="9" t="n">
+      <c r="Q9" s="8" t="n">
         <v>263000000</v>
       </c>
-      <c r="R9" s="9" t="n">
+      <c r="R9" s="8" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q9),ISNUMBER(M9),M9&gt;0),Q9/M9,"")</f>
         <v>255315.017959421</v>
       </c>
@@ -1472,46 +1629,46 @@
         <v>2630000</v>
       </c>
       <c r="U9" s="4" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="V9" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="W9" s="4"/>
       <c r="X9" s="4" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="Y9" s="4"/>
       <c r="Z9" s="4" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="AA9" s="4"/>
       <c r="AB9" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AC9" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AD9" s="4" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="AE9" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="AF9" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="AG9" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="AF9" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="AG9" s="4" t="s">
-        <v>64</v>
-      </c>
       <c r="AH9" s="4" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="AI9" s="4" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="AJ9" s="4" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1519,34 +1676,34 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>9</v>
@@ -1556,15 +1713,15 @@
       </c>
       <c r="N10" s="7"/>
       <c r="O10" s="4" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="Q10" s="9" t="n">
+      <c r="Q10" s="8" t="n">
         <v>17225000</v>
       </c>
-      <c r="R10" s="9" t="n">
+      <c r="R10" s="8" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q10),ISNUMBER(M10),M10&gt;0),Q10/M10,"")</f>
         <v>1314885.49618321</v>
       </c>
@@ -1575,50 +1732,50 @@
         <v>861250</v>
       </c>
       <c r="U10" s="4" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="V10" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="X10" s="4" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="Y10" s="4"/>
       <c r="Z10" s="4" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="AA10" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="AB10" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AC10" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AD10" s="4" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="AE10" s="4" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="AF10" s="4" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="AG10" s="4" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="AH10" s="4" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="AI10" s="4" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="AJ10" s="4" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1626,34 +1783,34 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="L11" s="4" t="n">
         <v>9</v>
@@ -1663,15 +1820,15 @@
       </c>
       <c r="N11" s="7"/>
       <c r="O11" s="4" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="P11" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q11" s="9" t="n">
+      <c r="Q11" s="8" t="n">
         <v>50797000</v>
       </c>
-      <c r="R11" s="9" t="n">
+      <c r="R11" s="8" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q11),ISNUMBER(M11),M11&gt;0),Q11/M11,"")</f>
         <v>303991.621783363</v>
       </c>
@@ -1682,47 +1839,47 @@
         <v>2539850</v>
       </c>
       <c r="U11" s="4" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="V11" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="X11" s="4" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="Y11" s="4"/>
       <c r="Z11" s="4" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="AA11" s="4" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="AB11" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AC11" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AD11" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AE11" s="4" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="AF11" s="4" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="AG11" s="4" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="AH11" s="4" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="AI11" s="4" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="AJ11" s="4"/>
     </row>
@@ -1731,34 +1888,34 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>113</v>
+        <v>41</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>114</v>
+        <v>62</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>4</v>
@@ -1773,10 +1930,10 @@
       <c r="P12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q12" s="9" t="n">
+      <c r="Q12" s="8" t="n">
         <v>195014000</v>
       </c>
-      <c r="R12" s="9" t="n">
+      <c r="R12" s="8" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q12),ISNUMBER(M12),M12&gt;0),Q12/M12,"")</f>
         <v>307399.117276166</v>
       </c>
@@ -1787,50 +1944,50 @@
         <v>1950140</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="V12" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="X12" s="4" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="Y12" s="4" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="Z12" s="4" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="AA12" s="4"/>
       <c r="AB12" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AC12" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AD12" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AE12" s="4" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="AF12" s="4" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="AG12" s="4" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="AH12" s="4" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="AI12" s="4" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="AJ12" s="4" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1838,34 +1995,34 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>113</v>
+        <v>41</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="L13" s="4" t="n">
         <v>12</v>
@@ -1880,10 +2037,10 @@
       <c r="P13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q13" s="9" t="n">
+      <c r="Q13" s="8" t="n">
         <v>158898000</v>
       </c>
-      <c r="R13" s="9" t="n">
+      <c r="R13" s="8" t="n">
         <f aca="false">IF(AND(ISNUMBER(Q13),ISNUMBER(M13),M13&gt;0),Q13/M13,"")</f>
         <v>176887.454079929</v>
       </c>
@@ -1894,114 +2051,117 @@
         <v>1588980</v>
       </c>
       <c r="U13" s="4" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="V13" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="X13" s="4" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="Y13" s="4" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="Z13" s="4" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="AA13" s="4"/>
       <c r="AB13" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AC13" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AD13" s="4" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="AE13" s="4" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="AF13" s="4" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="AG13" s="4" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="AH13" s="4" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="AI13" s="4" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="AJ13" s="4" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J14" s="10" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="M14" s="11" t="n">
         <f aca="false">SUM(M5:M13)</f>
-        <v>3216.5</v>
+        <v>4791.3</v>
       </c>
       <c r="Q14" s="12" t="n">
         <f aca="false">SUM(Q5:Q13)</f>
-        <v>939845000</v>
+        <v>1342354981</v>
       </c>
       <c r="R14" s="12" t="n">
         <f aca="false">IFERROR(SUM(Q5:Q13)/SUMIF(Q5:Q13,"&gt;0",M5:M13),"")</f>
-        <v>292194.932379916</v>
+        <v>280165.086928391</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:AJ13"/>
   <hyperlinks>
-    <hyperlink ref="C5" r:id="rId1" display="открыть"/>
-    <hyperlink ref="C6" r:id="rId2" display="открыть"/>
-    <hyperlink ref="C7" r:id="rId3" display="открыть"/>
-    <hyperlink ref="V7" r:id="rId4" display="roseltorg"/>
-    <hyperlink ref="W7" r:id="rId5" display="извещение"/>
-    <hyperlink ref="C8" r:id="rId6" display="открыть"/>
-    <hyperlink ref="V8" r:id="rId7" display="roseltorg"/>
-    <hyperlink ref="W8" r:id="rId8" display="извещение"/>
-    <hyperlink ref="C9" r:id="rId9" display="открыть"/>
-    <hyperlink ref="V9" r:id="rId10" display="roseltorg"/>
-    <hyperlink ref="C10" r:id="rId11" display="открыть"/>
-    <hyperlink ref="V10" r:id="rId12" display="roseltorg"/>
-    <hyperlink ref="W10" r:id="rId13" display="извещение"/>
-    <hyperlink ref="C11" r:id="rId14" display="открыть"/>
-    <hyperlink ref="V11" r:id="rId15" display="roseltorg"/>
-    <hyperlink ref="W11" r:id="rId16" display="извещение"/>
-    <hyperlink ref="C12" r:id="rId17" display="открыть"/>
-    <hyperlink ref="V12" r:id="rId18" display="roseltorg"/>
-    <hyperlink ref="W12" r:id="rId19" display="извещение"/>
-    <hyperlink ref="C13" r:id="rId20" display="открыть"/>
-    <hyperlink ref="V13" r:id="rId21" display="roseltorg"/>
-    <hyperlink ref="W13" r:id="rId22" display="извещение"/>
+    <hyperlink ref="C5" r:id="rId2" display="открыть"/>
+    <hyperlink ref="V5" r:id="rId3" display="roseltorg"/>
+    <hyperlink ref="W5" r:id="rId4" display="извещение"/>
+    <hyperlink ref="C6" r:id="rId5" display="открыть"/>
+    <hyperlink ref="V6" r:id="rId6" display="roseltorg"/>
+    <hyperlink ref="C7" r:id="rId7" display="открыть"/>
+    <hyperlink ref="V7" r:id="rId8" display="roseltorg"/>
+    <hyperlink ref="W7" r:id="rId9" display="извещение"/>
+    <hyperlink ref="C8" r:id="rId10" display="открыть"/>
+    <hyperlink ref="V8" r:id="rId11" display="roseltorg"/>
+    <hyperlink ref="W8" r:id="rId12" display="извещение"/>
+    <hyperlink ref="C9" r:id="rId13" display="открыть"/>
+    <hyperlink ref="V9" r:id="rId14" display="roseltorg"/>
+    <hyperlink ref="C10" r:id="rId15" display="открыть"/>
+    <hyperlink ref="V10" r:id="rId16" display="roseltorg"/>
+    <hyperlink ref="W10" r:id="rId17" display="извещение"/>
+    <hyperlink ref="C11" r:id="rId18" display="открыть"/>
+    <hyperlink ref="V11" r:id="rId19" display="roseltorg"/>
+    <hyperlink ref="W11" r:id="rId20" display="извещение"/>
+    <hyperlink ref="C12" r:id="rId21" display="открыть"/>
+    <hyperlink ref="V12" r:id="rId22" display="roseltorg"/>
+    <hyperlink ref="W12" r:id="rId23" display="извещение"/>
+    <hyperlink ref="C13" r:id="rId24" display="открыть"/>
+    <hyperlink ref="V13" r:id="rId25" display="roseltorg"/>
+    <hyperlink ref="W13" r:id="rId26" display="извещение"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2010,6 +2170,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId23"/>
+  <drawing r:id="rId27"/>
+  <legacyDrawing r:id="rId28"/>
 </worksheet>
 </file>
</xml_diff>